<commit_message>
Quita teléfono, fecha de envío y visto bueno del formato de las áreas
El consolidador y la app de escritorio ya no leen esos campos. Cuando un área
reenvía el formato, vale el archivo con la fecha de modificación más reciente.
</commit_message>
<xml_diff>
--- a/herramientas/plantilla/Formato Calendario Institucional - Areas.xlsx
+++ b/herramientas/plantilla/Formato Calendario Institucional - Areas.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ninchaustegui\Desktop\calendario_istitucional_Ucundinamrca\herramientas\plantilla\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DD035B4-9E06-423F-867E-6AE101D3F813}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DDE93A1-AB54-4E78-A8F7-BE5FECF860EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="390" yWindow="390" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Formato" sheetId="3" r:id="rId1"/>
@@ -201,7 +201,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="158">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="155">
   <si>
     <t>Formato de programación – Calendario Institucional</t>
   </si>
@@ -219,15 +219,6 @@
   </si>
   <si>
     <t>Correo institucional *</t>
-  </si>
-  <si>
-    <t>Extensión / teléfono</t>
-  </si>
-  <si>
-    <t>Fecha de envío</t>
-  </si>
-  <si>
-    <t>Visto bueno del jefe del área (nombre y cargo) *</t>
   </si>
   <si>
     <t>Actividades escritas</t>
@@ -835,7 +826,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -881,25 +872,13 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center"/>
       <protection locked="0"/>
     </xf>
@@ -910,6 +889,11 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1292,36 +1276,36 @@
     </row>
     <row r="2" spans="1:35" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
     </row>
     <row r="3" spans="1:35" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
     </row>
     <row r="4" spans="1:35" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="19"/>
-      <c r="C4" s="20"/>
-      <c r="D4" s="21" t="s">
+      <c r="B4" s="21"/>
+      <c r="C4" s="26"/>
+      <c r="D4" s="19" t="s">
         <v>4</v>
       </c>
-      <c r="E4" s="22"/>
-      <c r="F4" s="19"/>
-      <c r="G4" s="25"/>
-      <c r="H4" s="25"/>
-      <c r="I4" s="25"/>
-      <c r="J4" s="26" t="s">
-        <v>9</v>
-      </c>
-      <c r="K4" s="27"/>
-      <c r="L4" s="28"/>
+      <c r="E4" s="20"/>
+      <c r="F4" s="21"/>
+      <c r="G4" s="22"/>
+      <c r="H4" s="22"/>
+      <c r="I4" s="22"/>
+      <c r="J4" s="23" t="s">
+        <v>6</v>
+      </c>
+      <c r="K4" s="24"/>
+      <c r="L4" s="25"/>
       <c r="M4" s="18">
         <f>COUNTIF($AB$11:$AB$310,"?*")</f>
         <v>0</v>
@@ -1331,21 +1315,21 @@
       <c r="A5" s="16" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="19"/>
-      <c r="C5" s="20"/>
-      <c r="D5" s="21" t="s">
+      <c r="B5" s="21"/>
+      <c r="C5" s="26"/>
+      <c r="D5" s="19" t="s">
         <v>5</v>
       </c>
-      <c r="E5" s="22"/>
-      <c r="F5" s="19"/>
-      <c r="G5" s="25"/>
-      <c r="H5" s="25"/>
-      <c r="I5" s="25"/>
-      <c r="J5" s="26" t="s">
-        <v>10</v>
-      </c>
-      <c r="K5" s="27"/>
-      <c r="L5" s="28"/>
+      <c r="E5" s="20"/>
+      <c r="F5" s="21"/>
+      <c r="G5" s="22"/>
+      <c r="H5" s="22"/>
+      <c r="I5" s="22"/>
+      <c r="J5" s="23" t="s">
+        <v>7</v>
+      </c>
+      <c r="K5" s="24"/>
+      <c r="L5" s="25"/>
       <c r="M5" s="18">
         <f>COUNTIF($M$11:$M$310,"⚠*")</f>
         <v>0</v>
@@ -1355,21 +1339,19 @@
       <c r="A6" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="19"/>
-      <c r="C6" s="20"/>
-      <c r="D6" s="21" t="s">
-        <v>6</v>
-      </c>
-      <c r="E6" s="22"/>
-      <c r="F6" s="19"/>
-      <c r="G6" s="25"/>
-      <c r="H6" s="25"/>
-      <c r="I6" s="25"/>
-      <c r="J6" s="26" t="s">
-        <v>11</v>
-      </c>
-      <c r="K6" s="27"/>
-      <c r="L6" s="28"/>
+      <c r="B6" s="21"/>
+      <c r="C6" s="26"/>
+      <c r="D6" s="27"/>
+      <c r="E6" s="27"/>
+      <c r="F6" s="27"/>
+      <c r="G6" s="27"/>
+      <c r="H6" s="27"/>
+      <c r="I6" s="27"/>
+      <c r="J6" s="23" t="s">
+        <v>8</v>
+      </c>
+      <c r="K6" s="24"/>
+      <c r="L6" s="25"/>
       <c r="M6" s="18">
         <f>SUM($AF$11:$AF$310)</f>
         <v>0</v>
@@ -1377,25 +1359,23 @@
     </row>
     <row r="7" spans="1:35" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="16" t="s">
-        <v>92</v>
-      </c>
-      <c r="B7" s="19"/>
-      <c r="C7" s="20"/>
-      <c r="D7" s="21" t="s">
-        <v>7</v>
-      </c>
-      <c r="E7" s="22"/>
-      <c r="F7" s="23"/>
-      <c r="G7" s="24"/>
-      <c r="H7" s="24"/>
-      <c r="I7" s="24"/>
-      <c r="J7" s="26" t="s">
-        <v>12</v>
-      </c>
-      <c r="K7" s="27"/>
-      <c r="L7" s="28"/>
+        <v>89</v>
+      </c>
+      <c r="B7" s="21"/>
+      <c r="C7" s="26"/>
+      <c r="D7" s="27"/>
+      <c r="E7" s="27"/>
+      <c r="F7" s="27"/>
+      <c r="G7" s="27"/>
+      <c r="H7" s="27"/>
+      <c r="I7" s="27"/>
+      <c r="J7" s="23" t="s">
+        <v>9</v>
+      </c>
+      <c r="K7" s="24"/>
+      <c r="L7" s="25"/>
       <c r="M7" s="18" t="str">
-        <f>IF((B4="")+(B5="")+(B6="")+(B7="")+(F4="")+(F5="")+(F8="")&gt;0,"Corrija: complete los datos del área marcados con *",IF(M4=0,"Aún no hay actividades",IF(M5&gt;0,"Corrija las filas marcadas con ⚠ en rojo","✔ Listo para enviar")))</f>
+        <f>IF((B4="")+(B5="")+(B6="")+(B7="")+(F4="")+(F5="")&gt;0,"Corrija: complete los datos del área marcados con *",IF(M4=0,"Aún no hay actividades",IF(M5&gt;0,"Corrija las filas marcadas con ⚠ en rojo","✔ Listo para enviar")))</f>
         <v>Corrija: complete los datos del área marcados con *</v>
       </c>
     </row>
@@ -1403,118 +1383,116 @@
       <c r="A8" s="17"/>
       <c r="B8" s="17"/>
       <c r="C8" s="17"/>
-      <c r="D8" s="21" t="s">
-        <v>8</v>
-      </c>
-      <c r="E8" s="22"/>
-      <c r="F8" s="19"/>
-      <c r="G8" s="25"/>
-      <c r="H8" s="25"/>
-      <c r="I8" s="25"/>
+      <c r="D8" s="27"/>
+      <c r="E8" s="27"/>
+      <c r="F8" s="27"/>
+      <c r="G8" s="27"/>
+      <c r="H8" s="27"/>
+      <c r="I8" s="27"/>
     </row>
     <row r="9" spans="1:35" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="10" spans="1:35" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="G10" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B10" s="6" t="s">
+      <c r="H10" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="C10" s="6" t="s">
-        <v>93</v>
-      </c>
-      <c r="D10" s="6" t="s">
-        <v>94</v>
-      </c>
-      <c r="E10" s="6" t="s">
-        <v>95</v>
-      </c>
-      <c r="F10" s="6" t="s">
+      <c r="I10" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="G10" s="6" t="s">
+      <c r="J10" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="H10" s="6" t="s">
+      <c r="K10" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="I10" s="6" t="s">
+      <c r="L10" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="J10" s="6" t="s">
+      <c r="M10" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="K10" s="6" t="s">
+      <c r="N10" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="L10" s="6" t="s">
+      <c r="O10" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="M10" s="7" t="s">
+      <c r="P10" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="N10" s="8" t="s">
+      <c r="Q10" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="O10" s="8" t="s">
+      <c r="R10" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="P10" s="8" t="s">
+      <c r="S10" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="Q10" s="8" t="s">
+      <c r="T10" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="R10" s="8" t="s">
+      <c r="U10" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="S10" s="8" t="s">
+      <c r="V10" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="T10" s="8" t="s">
+      <c r="W10" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="U10" s="8" t="s">
+      <c r="X10" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="V10" s="8" t="s">
+      <c r="Y10" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="W10" s="8" t="s">
+      <c r="Z10" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="X10" s="8" t="s">
+      <c r="AB10" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="Y10" s="8" t="s">
+      <c r="AC10" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="Z10" s="6" t="s">
+      <c r="AD10" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="AB10" s="4" t="s">
+      <c r="AE10" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="AC10" s="4" t="s">
+      <c r="AF10" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="AD10" s="4" t="s">
+      <c r="AG10" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="AE10" s="4" t="s">
+      <c r="AH10" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="AF10" s="4" t="s">
+      <c r="AI10" s="4" t="s">
         <v>40</v>
-      </c>
-      <c r="AG10" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="AH10" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="AI10" s="4" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="11" spans="1:35" x14ac:dyDescent="0.25">
@@ -20420,25 +20398,19 @@
   </sheetData>
   <sheetProtection sheet="1" objects="1" scenarios="1" formatColumns="0" formatRows="0" autoFilter="0"/>
   <autoFilter ref="A10:Z310" xr:uid="{00000000-0009-0000-0000-000002000000}"/>
-  <mergeCells count="18">
-    <mergeCell ref="F7:I7"/>
-    <mergeCell ref="D8:E8"/>
-    <mergeCell ref="F8:I8"/>
+  <mergeCells count="12">
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="D5:E5"/>
     <mergeCell ref="J4:L4"/>
     <mergeCell ref="J5:L5"/>
     <mergeCell ref="J6:L6"/>
     <mergeCell ref="J7:L7"/>
     <mergeCell ref="F4:I4"/>
     <mergeCell ref="F5:I5"/>
-    <mergeCell ref="F6:I6"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="D5:E5"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="D7:E7"/>
   </mergeCells>
   <conditionalFormatting sqref="M11:M310">
     <cfRule type="expression" dxfId="4" priority="3" stopIfTrue="1">
@@ -20515,42 +20487,42 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D1" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="E1" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="F1" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="D1" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>61</v>
-      </c>
       <c r="G1" s="15" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="H1" s="15" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="E2" s="14">
         <v>46023</v>
@@ -20559,24 +20531,24 @@
         <v>0</v>
       </c>
       <c r="G2" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="H2" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="E3" s="14">
         <v>46034</v>
@@ -20585,24 +20557,24 @@
         <v>1</v>
       </c>
       <c r="G3" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="H3" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="E4" s="14">
         <v>46104</v>
@@ -20611,18 +20583,18 @@
         <v>2</v>
       </c>
       <c r="H4" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="E5" s="14">
         <v>46114</v>
@@ -20631,18 +20603,18 @@
         <v>3</v>
       </c>
       <c r="H5" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="E6" s="14">
         <v>46115</v>
@@ -20651,18 +20623,18 @@
         <v>4</v>
       </c>
       <c r="H6" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="E7" s="14">
         <v>46143</v>
@@ -20671,18 +20643,18 @@
         <v>5</v>
       </c>
       <c r="H7" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="E8" s="14">
         <v>46160</v>
@@ -20691,18 +20663,18 @@
         <v>6</v>
       </c>
       <c r="H8" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="E9" s="14">
         <v>46181</v>
@@ -20711,15 +20683,15 @@
         <v>7</v>
       </c>
       <c r="H9" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="E10" s="14">
         <v>46188</v>
@@ -20728,12 +20700,12 @@
         <v>8</v>
       </c>
       <c r="H10" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="E11" s="14">
         <v>46202</v>
@@ -20742,12 +20714,12 @@
         <v>9</v>
       </c>
       <c r="H11" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="E12" s="14">
         <v>46223</v>
@@ -20756,12 +20728,12 @@
         <v>10</v>
       </c>
       <c r="H12" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="E13" s="14">
         <v>46241</v>
@@ -20770,12 +20742,12 @@
         <v>11</v>
       </c>
       <c r="H13" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="E14" s="14">
         <v>46251</v>
@@ -20784,12 +20756,12 @@
         <v>12</v>
       </c>
       <c r="H14" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="E15" s="14">
         <v>46307</v>
@@ -20798,12 +20770,12 @@
         <v>13</v>
       </c>
       <c r="H15" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="E16" s="14">
         <v>46328</v>
@@ -20812,12 +20784,12 @@
         <v>14</v>
       </c>
       <c r="H16" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="E17" s="14">
         <v>46342</v>
@@ -20826,12 +20798,12 @@
         <v>15</v>
       </c>
       <c r="H17" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="E18" s="14">
         <v>46364</v>
@@ -20840,12 +20812,12 @@
         <v>16</v>
       </c>
       <c r="H18" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="E19" s="14">
         <v>46381</v>
@@ -20854,12 +20826,12 @@
         <v>17</v>
       </c>
       <c r="H19" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="E20" s="14">
         <v>46388</v>
@@ -20868,7 +20840,7 @@
         <v>18</v>
       </c>
       <c r="H20" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
@@ -20879,7 +20851,7 @@
         <v>19</v>
       </c>
       <c r="H21" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
@@ -20890,7 +20862,7 @@
         <v>20</v>
       </c>
       <c r="H22" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
@@ -20901,7 +20873,7 @@
         <v>21</v>
       </c>
       <c r="H23" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
@@ -20912,7 +20884,7 @@
         <v>22</v>
       </c>
       <c r="H24" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
@@ -20923,7 +20895,7 @@
         <v>23</v>
       </c>
       <c r="H25" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
@@ -20934,7 +20906,7 @@
         <v>24</v>
       </c>
       <c r="H26" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
@@ -20945,7 +20917,7 @@
         <v>25</v>
       </c>
       <c r="H27" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
@@ -20956,7 +20928,7 @@
         <v>26</v>
       </c>
       <c r="H28" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
@@ -20967,7 +20939,7 @@
         <v>27</v>
       </c>
       <c r="H29" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
@@ -20978,7 +20950,7 @@
         <v>28</v>
       </c>
       <c r="H30" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.25">
@@ -20989,7 +20961,7 @@
         <v>29</v>
       </c>
       <c r="H31" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
@@ -21000,7 +20972,7 @@
         <v>30</v>
       </c>
       <c r="H32" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
     </row>
     <row r="33" spans="5:8" x14ac:dyDescent="0.25">
@@ -21011,7 +20983,7 @@
         <v>31</v>
       </c>
       <c r="H33" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
     </row>
     <row r="34" spans="5:8" x14ac:dyDescent="0.25">
@@ -21022,7 +20994,7 @@
         <v>32</v>
       </c>
       <c r="H34" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
     </row>
     <row r="35" spans="5:8" x14ac:dyDescent="0.25">
@@ -21033,7 +21005,7 @@
         <v>33</v>
       </c>
       <c r="H35" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
     </row>
     <row r="36" spans="5:8" x14ac:dyDescent="0.25">
@@ -21044,7 +21016,7 @@
         <v>34</v>
       </c>
       <c r="H36" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
     </row>
     <row r="37" spans="5:8" x14ac:dyDescent="0.25">
@@ -21055,7 +21027,7 @@
         <v>35</v>
       </c>
       <c r="H37" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
     </row>
     <row r="38" spans="5:8" x14ac:dyDescent="0.25">
@@ -21066,7 +21038,7 @@
         <v>36</v>
       </c>
       <c r="H38" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
     </row>
     <row r="39" spans="5:8" x14ac:dyDescent="0.25">
@@ -21077,7 +21049,7 @@
         <v>37</v>
       </c>
       <c r="H39" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
     </row>
     <row r="40" spans="5:8" x14ac:dyDescent="0.25">
@@ -21088,7 +21060,7 @@
         <v>38</v>
       </c>
       <c r="H40" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
     </row>
     <row r="41" spans="5:8" x14ac:dyDescent="0.25">
@@ -21099,7 +21071,7 @@
         <v>39</v>
       </c>
       <c r="H41" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
     </row>
     <row r="42" spans="5:8" x14ac:dyDescent="0.25">
@@ -21110,7 +21082,7 @@
         <v>40</v>
       </c>
       <c r="H42" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
     </row>
     <row r="43" spans="5:8" x14ac:dyDescent="0.25">
@@ -21121,7 +21093,7 @@
         <v>41</v>
       </c>
       <c r="H43" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
     </row>
     <row r="44" spans="5:8" x14ac:dyDescent="0.25">
@@ -21132,7 +21104,7 @@
         <v>42</v>
       </c>
       <c r="H44" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
     </row>
     <row r="45" spans="5:8" x14ac:dyDescent="0.25">
@@ -21143,7 +21115,7 @@
         <v>43</v>
       </c>
       <c r="H45" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
     </row>
     <row r="46" spans="5:8" x14ac:dyDescent="0.25">
@@ -21154,7 +21126,7 @@
         <v>44</v>
       </c>
       <c r="H46" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
     </row>
     <row r="47" spans="5:8" x14ac:dyDescent="0.25">
@@ -21165,7 +21137,7 @@
         <v>45</v>
       </c>
       <c r="H47" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
     </row>
     <row r="48" spans="5:8" x14ac:dyDescent="0.25">
@@ -21176,7 +21148,7 @@
         <v>46</v>
       </c>
       <c r="H48" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
     </row>
     <row r="49" spans="5:8" x14ac:dyDescent="0.25">
@@ -21187,7 +21159,7 @@
         <v>47</v>
       </c>
       <c r="H49" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
     </row>
     <row r="50" spans="5:8" x14ac:dyDescent="0.25">
@@ -21198,7 +21170,7 @@
         <v>48</v>
       </c>
       <c r="H50" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
     </row>
     <row r="51" spans="5:8" x14ac:dyDescent="0.25">
@@ -21209,7 +21181,7 @@
         <v>49</v>
       </c>
       <c r="H51" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
     </row>
     <row r="52" spans="5:8" x14ac:dyDescent="0.25">
@@ -21220,7 +21192,7 @@
         <v>50</v>
       </c>
       <c r="H52" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
     </row>
     <row r="53" spans="5:8" x14ac:dyDescent="0.25">
@@ -21231,7 +21203,7 @@
         <v>51</v>
       </c>
       <c r="H53" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
     </row>
     <row r="54" spans="5:8" x14ac:dyDescent="0.25">
@@ -21242,7 +21214,7 @@
         <v>52</v>
       </c>
       <c r="H54" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
     </row>
     <row r="55" spans="5:8" x14ac:dyDescent="0.25">
@@ -21253,7 +21225,7 @@
         <v>53</v>
       </c>
       <c r="H55" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
     </row>
     <row r="56" spans="5:8" x14ac:dyDescent="0.25">
@@ -21261,7 +21233,7 @@
         <v>54</v>
       </c>
       <c r="H56" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="57" spans="5:8" x14ac:dyDescent="0.25">
@@ -21269,7 +21241,7 @@
         <v>55</v>
       </c>
       <c r="H57" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
     </row>
     <row r="58" spans="5:8" x14ac:dyDescent="0.25">
@@ -21277,7 +21249,7 @@
         <v>56</v>
       </c>
       <c r="H58" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
     </row>
     <row r="59" spans="5:8" x14ac:dyDescent="0.25">
@@ -21285,7 +21257,7 @@
         <v>57</v>
       </c>
       <c r="H59" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
     </row>
     <row r="60" spans="5:8" x14ac:dyDescent="0.25">
@@ -21293,7 +21265,7 @@
         <v>58</v>
       </c>
       <c r="H60" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
     </row>
     <row r="61" spans="5:8" x14ac:dyDescent="0.25">
@@ -21301,7 +21273,7 @@
         <v>59</v>
       </c>
       <c r="H61" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
     </row>
     <row r="62" spans="5:8" x14ac:dyDescent="0.25">
@@ -21309,7 +21281,7 @@
         <v>60</v>
       </c>
       <c r="H62" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
     </row>
     <row r="63" spans="5:8" x14ac:dyDescent="0.25">

</xml_diff>